<commit_message>
Add day tabs to Excel schedule
</commit_message>
<xml_diff>
--- a/output/barn_schedule.xlsx
+++ b/output/barn_schedule.xlsx
@@ -7,11 +7,20 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Barn Schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Rides" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fri" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sat" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sun" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Barn Schedule'!$A$1:$J$27</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Barn Schedule'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Rides'!$A$1:$J$27</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Rides'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fri'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Fri'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sat'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sat'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sun'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Sun'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,9 +456,9 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1654,4 +1663,1388 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>7:45 AM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Franzsis HSR</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1FI2EF</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>FEI Intermediate II Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>8:55 AM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Vholt</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1PSG</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>FEI Prix St. Georges</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Roberts Arena (Beverly Rogers at C)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>8:56 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Gillman, Chynna</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Destemido RRI</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>H1PSG</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>FEI Prix. St. Georges</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Jodi Lees at C)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>10:09 AM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Steendieks Dubidoo</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>H1PSG</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>FEI Prix. St. Georges</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Jodi Lees at C)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>11:05 AM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Matchmaker HSR</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Third Level Test 3</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Jumper Ring (Jodi Ely at C)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>11:37 AM</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Kuhn, Malcolm</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Moon</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>H1UB</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>USDF Introductory Test B</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>1:20 PM</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Gillman, Chynna</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Padme Zarma TF</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Second Level Test 1</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Jumper Ring (Jodi Ely at C)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Va Fiero</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>1T3</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Training Level Test 3</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 2 (Joan Williams at C)</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>5:46 PM</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Wilton, Jordan</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Wild Card HSR</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>1FFS</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>FEI Freestyle Test of Choice</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Roberts Arena (Beverly Rogers at C)</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Fiorenza HSR</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Second Level Test 3</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>8:22 AM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Gillman, Chynna</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Destemido RRI</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>H2PSG</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>FEI Prix St. Georges</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>9:45 AM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Steendieks Dubidoo</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>H2I1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>FEI Intermediare I</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>12:51 PM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Fiorenza HSR</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Third Level Test 3</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1:13 PM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Kuhn, Malcolm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Moon</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>H2UC</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>USDF Introductory Test C</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1:50 PM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Gillman, Chynna</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Padme Zarma TF</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>First Level Test 3</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2:49 PM</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Vholt</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2I1</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>FEI Intermediare I</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2:58 PM</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Wilton, Jordan</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Wild Card HSR</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2I1</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>FEI Intermediare I</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3:47 PM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Matchmaker HSR</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Third Level Test 3</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>4:37 PM</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Franzsis HSR</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2I2</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>FEI Intermediare II</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>6:33 PM</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Va Fiero</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2YH</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Young Horse Test of Choice (excl 7YO)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Roberts Arena (Jodi Ely at C)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>7:30 AM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Va Fiero</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>US4EF</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>8:31 AM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Franzsis HSR</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>DHGEF</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>USEF Developing Horse Grand Prix Test Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>9:29 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Matchmaker HSR</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Third Level Test 3</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Christel Carlson at C)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>10:37 AM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Fiorenza HSR</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Third Level Test 3</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Hunter 1 (Christel Carlson at C)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>12:56 PM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Vholt</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>3PSG</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>FEI Prix St. Georges</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1:27 PM</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Wilton, Jordan</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Wild Card HSR</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>3FFS</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>FEI Freestyle Test of Choice</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add printable sheet titles
</commit_message>
<xml_diff>
--- a/output/barn_schedule.xlsx
+++ b/output/barn_schedule.xlsx
@@ -13,14 +13,14 @@
     <sheet name="Sun" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Rides'!$A$1:$J$27</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Rides'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fri'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Fri'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sat'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sat'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sun'!$A$1:$J$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Sun'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Rides'!$A$3:$J$29</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Rides'!$1:$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fri'!$A$3:$J$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Fri'!$1:$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sat'!$A$3:$J$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sat'!$1:$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sun'!$A$3:$J$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Sun'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,13 +29,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
@@ -71,9 +75,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -447,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -462,1204 +469,1214 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ride Time</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ready By / On Horse By</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Rider</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Horse</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Class #</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Class Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Arena #</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Arena Name</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>7:45 AM</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Franzsis HSR</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>1FI2EF</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>FEI Intermediate II Markel/USEF Qualifying</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>All Rides Barn Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>7:45 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Franzsis HSR</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>1FI2EF</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>FEI Intermediate II Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>8:55 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>1PSG</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>8:56 AM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>10:09 AM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>11:05 AM</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>133</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>11:37 AM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>H1UB</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test B</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>1:20 PM</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>121</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 1</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>5:46 PM</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>1FFS</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>8:22 AM</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>H2PSG</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>9:45 AM</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>H2I1</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>12:51 PM</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>1:13 PM</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>H2UC</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test C</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>1:50 PM</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>2:49 PM</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>2:58 PM</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>3:47 PM</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>4:37 PM</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>2I2</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare II</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>6:33 PM</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>2YH</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Young Horse Test of Choice (excl 7YO)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>7:30 AM</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>US4EF</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>8:31 AM</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>DHGEF</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>USEF Developing Horse Grand Prix Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>9:29 AM</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>10:37 AM</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>12:56 PM</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>3PSG</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>1:27 PM</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>3FFS</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J27"/>
+  <autoFilter ref="A3:J29"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1671,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1686,500 +1703,510 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ride Time</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ready By / On Horse By</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Rider</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Horse</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Class #</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Class Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Arena #</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Arena Name</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>7:45 AM</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Franzsis HSR</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>1FI2EF</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>FEI Intermediate II Markel/USEF Qualifying</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>Friday Barn Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>7:45 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Franzsis HSR</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>1FI2EF</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>FEI Intermediate II Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>8:55 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>1PSG</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>8:56 AM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>10:09 AM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>11:05 AM</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>133</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>11:37 AM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>H1UB</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test B</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>1:20 PM</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>121</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 1</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>5:46 PM</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>1FFS</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J11"/>
+  <autoFilter ref="A3:J13"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2191,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2206,500 +2233,510 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ride Time</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ready By / On Horse By</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Rider</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Horse</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Class #</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Class Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Arena #</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Arena Name</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>8:22 AM</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Gillman, Chynna</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Destemido RRI</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>H2PSG</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>FEI Prix St. Georges</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R &amp; L Arena (Susan Mandas at C)</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>Saturday Barn Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>8:22 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Gillman, Chynna</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Destemido RRI</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>H2PSG</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>FEI Prix St. Georges</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Susan Mandas at C)</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>9:45 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>H2I1</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>12:51 PM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>1:13 PM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>H2UC</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test C</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>1:50 PM</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>2:49 PM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2:58 PM</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>3:47 PM</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>4:37 PM</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>2I2</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare II</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>6:33 PM</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>2YH</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Young Horse Test of Choice (excl 7YO)</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J11"/>
+  <autoFilter ref="A3:J13"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2711,7 +2748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2726,324 +2763,334 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ride Time</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Ready By / On Horse By</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Rider</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Horse</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Class #</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Class Name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Arena #</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Arena Name</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>7:30 AM</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Va Fiero</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>US4EF</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>Sunday Barn Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ride Time</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ready By / On Horse By</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Class #</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Arena #</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Arena Name</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>7:30 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Va Fiero</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>US4EF</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>8:31 AM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>DHGEF</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>USEF Developing Horse Grand Prix Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>9:29 AM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>10:37 AM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>12:56 PM</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Fleming-Kuhn, Kathryn</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Fleming-Kuhn, Kathryn</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>3PSG</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>1:27 PM</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>3FFS</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A3:J9"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>